<commit_message>
Add cards-timeline block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/cards-timeline/cards-timeline.css
- blocks/cards-timeline/cards-timeline.js
- tools/importer/import-standalone.bundle.js
- tools/importer/import-standalone.js
- tools/importer/page-templates.json
- tools/importer/parsers/cards-article.js
- tools/importer/parsers/cards-timeline.js
- tools/importer/reports/about.report.json
- tools/importer/reports/import-standalone.report.xlsx
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-standalone.report.xlsx
+++ b/tools/importer/reports/import-standalone.report.xlsx
@@ -40,7 +40,7 @@
     <t>about.report.json</t>
   </si>
   <si>
-    <t>["cards-article"]</t>
+    <t>["cards-timeline"]</t>
   </si>
   <si>
     <t>about</t>
@@ -52,7 +52,7 @@
     <t>standalone</t>
   </si>
   <si>
-    <t>2026-06-28T17:49:20.218Z</t>
+    <t>2026-06-29T05:06:54.954Z</t>
   </si>
   <si>
     <t>About Us | MOOG Parts</t>

</xml_diff>